<commit_message>
Add vmp reverse blog
</commit_message>
<xml_diff>
--- a/vmp_reverse/栈.xlsx
+++ b/vmp_reverse/栈.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255" activeTab="4"/>
+    <workbookView windowWidth="28800" windowHeight="12255" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="环境恢复前" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="46">
   <si>
     <t>ThreadId</t>
   </si>
@@ -815,11 +815,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1346,270 +1346,270 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="E11:N40"/>
+  <dimension ref="B2:K31"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="5" max="5" width="17.625" customWidth="1"/>
-    <col min="8" max="8" width="11.375" customWidth="1"/>
-    <col min="11" max="11" width="10.375" customWidth="1"/>
-    <col min="12" max="12" width="16.375" customWidth="1"/>
-    <col min="13" max="13" width="8" customWidth="1"/>
-    <col min="14" max="14" width="24.25" customWidth="1"/>
+    <col min="2" max="2" width="17.625" customWidth="1"/>
+    <col min="5" max="5" width="11.375" customWidth="1"/>
+    <col min="8" max="8" width="10.375" customWidth="1"/>
+    <col min="9" max="9" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="24.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="6:8">
-      <c r="G11">
+    <row r="2" spans="3:5">
+      <c r="D2">
         <v>0</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="6:8">
-      <c r="F12" t="s">
+    <row r="3" spans="3:5">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="G12">
+      <c r="D3">
         <v>4</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="6:8">
-      <c r="H13" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="6:8">
-      <c r="H14" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="6:8">
-      <c r="H15" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="6:8">
-      <c r="H16" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="5:14">
-      <c r="H17" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="5:14">
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="5:14">
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="5:14">
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="5:14">
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="5:14">
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="5:14">
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="5:14">
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" spans="5:14">
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" spans="5:14">
-      <c r="E26" t="s">
+      <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5">
+      <c r="E4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5">
+      <c r="E5" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5">
+      <c r="E6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5">
+      <c r="E7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5">
+      <c r="E8" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5">
+      <c r="E9" s="1"/>
+    </row>
+    <row r="10" spans="3:5">
+      <c r="E10" s="1"/>
+    </row>
+    <row r="11" spans="3:5">
+      <c r="E11" s="1"/>
+    </row>
+    <row r="12" spans="3:5">
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" spans="3:5">
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" spans="3:5">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="3:5">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="3:5">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="2:11">
+      <c r="B17" t="s">
         <v>3</v>
       </c>
-      <c r="F26" t="s">
+      <c r="C17" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="2">
+      <c r="D17" s="2">
         <v>0</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="E17" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L26" t="s">
+      <c r="I17" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="5:14">
-      <c r="G27" s="2">
+    <row r="18" spans="2:11">
+      <c r="D18" s="2">
         <v>1</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="E18" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L27" t="s">
+      <c r="I18" t="s">
         <v>8</v>
       </c>
-      <c r="M27" s="4">
+      <c r="J18" s="3">
         <v>0</v>
       </c>
-      <c r="N27" t="s">
+      <c r="K18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="5:14">
-      <c r="G28" s="2">
-        <v>2</v>
-      </c>
-      <c r="H28" s="3"/>
-      <c r="M28" s="4">
+    <row r="19" spans="2:11">
+      <c r="D19" s="2">
+        <v>2</v>
+      </c>
+      <c r="E19" s="4"/>
+      <c r="J19" s="3">
         <v>4</v>
       </c>
-      <c r="N28" t="s">
+      <c r="K19" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="5:14">
-      <c r="G29" s="2">
+    <row r="20" spans="2:11">
+      <c r="D20" s="2">
         <v>3</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M29" s="4">
+      <c r="J20" s="3">
         <v>8</v>
       </c>
-      <c r="N29" t="s">
+      <c r="K20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="5:14">
-      <c r="G30" s="2">
+    <row r="21" spans="2:11">
+      <c r="D21" s="2">
         <v>4</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="J21" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N30" t="s">
+      <c r="K21" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="5:14">
-      <c r="G31" s="2">
+    <row r="22" spans="2:11">
+      <c r="D22" s="2">
         <v>5</v>
       </c>
-      <c r="H31" s="3"/>
-      <c r="M31" s="4">
+      <c r="E22" s="4"/>
+      <c r="J22" s="3">
         <v>10</v>
       </c>
-      <c r="N31" t="s">
+      <c r="K22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="5:14">
-      <c r="G32" s="2">
+    <row r="23" spans="2:11">
+      <c r="D23" s="2">
         <v>6</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="M32" s="4">
+      <c r="J23" s="3">
         <v>14</v>
       </c>
-      <c r="N32" t="s">
+      <c r="K23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="33" spans="7:14">
-      <c r="G33" s="2">
+    <row r="24" spans="2:11">
+      <c r="D24" s="2">
         <v>7</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="M33" s="4">
+      <c r="J24" s="3">
         <v>18</v>
       </c>
-      <c r="N33" t="s">
+      <c r="K24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="7:14">
-      <c r="G34" s="2">
+    <row r="25" spans="2:11">
+      <c r="D25" s="2">
         <v>8</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="M34" s="4" t="s">
+      <c r="E25" s="4"/>
+      <c r="J25" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N34" t="s">
+      <c r="K25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="7:14">
-      <c r="G35" s="2">
+    <row r="26" spans="2:11">
+      <c r="D26" s="2">
         <v>9</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="E26" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="M35" s="4">
+      <c r="J26" s="3">
         <v>20</v>
       </c>
-      <c r="N35" t="s">
+      <c r="K26" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="7:14">
-      <c r="G36" s="2" t="s">
+    <row r="27" spans="2:11">
+      <c r="D27" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="M36" s="4">
+      <c r="J27" s="3">
         <v>24</v>
       </c>
-      <c r="N36" t="s">
+      <c r="K27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="7:14">
-      <c r="G37" s="2" t="s">
+    <row r="28" spans="2:11">
+      <c r="D28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H37" s="3"/>
-      <c r="M37" s="4">
+      <c r="E28" s="4"/>
+      <c r="J28" s="3">
         <v>28</v>
       </c>
-      <c r="N37" t="s">
+      <c r="K28" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="7:14">
-      <c r="G38" s="2" t="s">
+    <row r="29" spans="2:11">
+      <c r="D29" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="E29" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="7:14">
-      <c r="G39" s="2" t="s">
+    <row r="30" spans="2:11">
+      <c r="D30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="3"/>
-    </row>
-    <row r="40" spans="7:14">
-      <c r="G40" s="2" t="s">
+      <c r="E30" s="4"/>
+    </row>
+    <row r="31" spans="2:11">
+      <c r="D31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="E31" s="4" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1622,274 +1622,274 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="E11:O40"/>
+  <dimension ref="B5:L34"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="5" max="5" width="17.625" customWidth="1"/>
-    <col min="8" max="8" width="11.375" customWidth="1"/>
-    <col min="11" max="11" width="10.375" customWidth="1"/>
-    <col min="12" max="12" width="16.375" customWidth="1"/>
-    <col min="13" max="13" width="8" customWidth="1"/>
-    <col min="14" max="14" width="11.625" customWidth="1"/>
-    <col min="15" max="15" width="13.125" customWidth="1"/>
+    <col min="2" max="2" width="17.625" customWidth="1"/>
+    <col min="5" max="5" width="11.375" customWidth="1"/>
+    <col min="8" max="8" width="10.375" customWidth="1"/>
+    <col min="9" max="9" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="11.625" customWidth="1"/>
+    <col min="12" max="12" width="13.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" customFormat="1" spans="6:8">
-      <c r="G11">
+    <row r="5" customFormat="1" spans="3:5">
+      <c r="D5">
         <v>0</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="6:8">
-      <c r="F12" t="s">
+    <row r="6" customFormat="1" spans="3:5">
+      <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="G12">
+      <c r="D6">
         <v>4</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" customFormat="1" spans="6:8">
-      <c r="H13" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" customFormat="1" spans="6:8">
-      <c r="H14" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" spans="6:8">
-      <c r="H15" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" customFormat="1" spans="6:8">
-      <c r="H16" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" customFormat="1" spans="5:14">
-      <c r="H17" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" customFormat="1" spans="5:14">
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" customFormat="1" spans="5:14">
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" customFormat="1" spans="5:14">
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" customFormat="1" spans="5:14">
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" customFormat="1" spans="5:14">
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" customFormat="1" spans="5:14">
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" customFormat="1" spans="5:14">
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" customFormat="1" spans="5:14">
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" customFormat="1" spans="5:14">
-      <c r="E26" t="s">
+      <c r="E6" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="1" spans="3:5">
+      <c r="E7" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="1" spans="3:5">
+      <c r="E8" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" spans="3:5">
+      <c r="E9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" customFormat="1" spans="3:5">
+      <c r="E10" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="1" spans="3:5">
+      <c r="E11" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="1" spans="3:5">
+      <c r="E12" s="1"/>
+    </row>
+    <row r="13" customFormat="1" spans="3:5">
+      <c r="E13" s="1"/>
+    </row>
+    <row r="14" customFormat="1" spans="3:5">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" customFormat="1" spans="3:5">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" customFormat="1" spans="3:5">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" customFormat="1" spans="2:12">
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" customFormat="1" spans="2:12">
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" customFormat="1" spans="2:12">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" customFormat="1" spans="2:12">
+      <c r="B20" t="s">
         <v>3</v>
       </c>
-      <c r="F26" t="s">
+      <c r="C20" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="2">
+      <c r="D20" s="2">
         <v>0</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="E20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="L26" t="s">
+      <c r="I20" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" customFormat="1" spans="5:14">
-      <c r="G27" s="2">
+    <row r="21" customFormat="1" spans="2:12">
+      <c r="D21" s="2">
         <v>1</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="E21" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="4">
+      <c r="J21" s="3">
         <v>0</v>
       </c>
-      <c r="N27" t="s">
+      <c r="K21" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" customFormat="1" spans="5:14">
-      <c r="G28" s="2">
-        <v>2</v>
-      </c>
-      <c r="H28" s="3"/>
-      <c r="M28" s="4">
+    <row r="22" customFormat="1" spans="2:12">
+      <c r="D22" s="2">
+        <v>2</v>
+      </c>
+      <c r="E22" s="4"/>
+      <c r="J22" s="3">
         <v>4</v>
       </c>
-      <c r="N28" t="s">
+      <c r="K22" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" customFormat="1" spans="5:14">
-      <c r="G29" s="2">
+    <row r="23" customFormat="1" spans="2:12">
+      <c r="D23" s="2">
         <v>3</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="E23" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="4">
+      <c r="J23" s="3">
         <v>8</v>
       </c>
-      <c r="N29" t="s">
+      <c r="K23" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" customFormat="1" spans="5:14">
-      <c r="G30" s="2">
+    <row r="24" customFormat="1" spans="2:12">
+      <c r="D24" s="2">
         <v>4</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="J24" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N30" t="s">
+      <c r="K24" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" customFormat="1" spans="5:14">
-      <c r="G31" s="2">
+    <row r="25" customFormat="1" spans="2:12">
+      <c r="D25" s="2">
         <v>5</v>
       </c>
-      <c r="H31" s="3"/>
-      <c r="M31" s="4">
+      <c r="E25" s="4"/>
+      <c r="J25" s="3">
         <v>10</v>
       </c>
-      <c r="N31" t="s">
+      <c r="K25" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" customFormat="1" spans="5:14">
-      <c r="G32" s="2">
+    <row r="26" customFormat="1" spans="2:12">
+      <c r="D26" s="2">
         <v>6</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="E26" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M32" s="4">
+      <c r="J26" s="3">
         <v>14</v>
       </c>
-      <c r="N32" t="s">
+      <c r="K26" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="33" customFormat="1" spans="7:15">
-      <c r="G33" s="2">
+    <row r="27" customFormat="1" spans="2:12">
+      <c r="D27" s="2">
         <v>7</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="M33" s="4">
+      <c r="J27" s="3">
         <v>18</v>
       </c>
-      <c r="N33" t="s">
+      <c r="K27" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" customFormat="1" spans="7:15">
-      <c r="G34" s="2">
+    <row r="28" customFormat="1" spans="2:12">
+      <c r="D28" s="2">
         <v>8</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="M34" s="4" t="s">
+      <c r="E28" s="4"/>
+      <c r="J28" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N34" t="s">
+      <c r="K28" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="35" customFormat="1" spans="7:15">
-      <c r="G35" s="2">
+    <row r="29" customFormat="1" spans="2:12">
+      <c r="D29" s="2">
         <v>9</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="E29" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M35" s="4">
+      <c r="J29" s="3">
         <v>20</v>
       </c>
-      <c r="N35" t="s">
+      <c r="K29" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" customFormat="1" spans="7:15">
-      <c r="G36" s="2" t="s">
+    <row r="30" customFormat="1" spans="2:12">
+      <c r="D30" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="E30" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M36" s="4">
+      <c r="J30" s="3">
         <v>24</v>
       </c>
-      <c r="N36" t="s">
+      <c r="K30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" customFormat="1" spans="7:15">
-      <c r="G37" s="2" t="s">
+    <row r="31" customFormat="1" spans="2:12">
+      <c r="D31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H37" s="3"/>
-      <c r="M37" s="4">
+      <c r="E31" s="4"/>
+      <c r="J31" s="3">
         <v>28</v>
       </c>
-      <c r="N37" t="s">
+      <c r="K31" t="s">
         <v>28</v>
       </c>
-      <c r="O37" t="s">
+      <c r="L31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="38" customFormat="1" spans="7:15">
-      <c r="G38" s="2" t="s">
+    <row r="32" customFormat="1" spans="2:12">
+      <c r="D32" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="E32" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L38" t="s">
+      <c r="I32" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="39" customFormat="1" spans="7:15">
-      <c r="G39" s="2" t="s">
+    <row r="33" customFormat="1" spans="4:5">
+      <c r="D33" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="3"/>
-    </row>
-    <row r="40" spans="7:15">
-      <c r="G40" s="2" t="s">
+      <c r="E33" s="4"/>
+    </row>
+    <row r="34" spans="4:5">
+      <c r="D34" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="E34" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1902,276 +1902,276 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="E11:O40"/>
+  <dimension ref="B8:L37"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="5" max="5" width="17.625" customWidth="1"/>
-    <col min="8" max="8" width="11.375" customWidth="1"/>
-    <col min="11" max="11" width="10.375" customWidth="1"/>
-    <col min="12" max="12" width="16.375" customWidth="1"/>
-    <col min="13" max="13" width="8" customWidth="1"/>
-    <col min="14" max="14" width="11.625" customWidth="1"/>
-    <col min="15" max="15" width="13.125" customWidth="1"/>
+    <col min="2" max="2" width="17.625" customWidth="1"/>
+    <col min="5" max="5" width="11.375" customWidth="1"/>
+    <col min="8" max="8" width="10.375" customWidth="1"/>
+    <col min="9" max="9" width="16.375" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="11.625" customWidth="1"/>
+    <col min="12" max="12" width="13.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" customFormat="1" spans="6:8">
-      <c r="G11">
+    <row r="8" customFormat="1" spans="3:5">
+      <c r="D8">
         <v>0</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" customFormat="1" spans="6:8">
-      <c r="F12" t="s">
+    <row r="9" customFormat="1" spans="3:5">
+      <c r="C9" t="s">
         <v>1</v>
       </c>
-      <c r="G12">
+      <c r="D9">
         <v>4</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" customFormat="1" spans="6:8">
-      <c r="H13" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" customFormat="1" spans="6:8">
-      <c r="H14" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" spans="6:8">
-      <c r="H15" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" customFormat="1" spans="6:8">
-      <c r="H16" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" customFormat="1" spans="5:14">
-      <c r="H17" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" customFormat="1" spans="5:14">
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" customFormat="1" spans="5:14">
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" customFormat="1" spans="5:14">
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" customFormat="1" spans="5:14">
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" customFormat="1" spans="5:14">
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" customFormat="1" spans="5:14">
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" customFormat="1" spans="5:14">
-      <c r="H24" s="1"/>
-    </row>
-    <row r="25" customFormat="1" spans="5:14">
-      <c r="H25" s="1"/>
-    </row>
-    <row r="26" customFormat="1" spans="5:14">
-      <c r="E26" t="s">
+      <c r="E9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" customFormat="1" spans="3:5">
+      <c r="E10" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="1" spans="3:5">
+      <c r="E11" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="1" spans="3:5">
+      <c r="E12" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" customFormat="1" spans="3:5">
+      <c r="E13" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" customFormat="1" spans="3:5">
+      <c r="E14" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" spans="3:5">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" customFormat="1" spans="3:5">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" customFormat="1" spans="2:11">
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" customFormat="1" spans="2:11">
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" customFormat="1" spans="2:11">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" customFormat="1" spans="2:11">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" customFormat="1" spans="2:11">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" customFormat="1" spans="2:11">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" customFormat="1" spans="2:11">
+      <c r="B23" t="s">
         <v>3</v>
       </c>
-      <c r="F26" t="s">
+      <c r="C23" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="2">
+      <c r="D23" s="2">
         <v>0</v>
       </c>
-      <c r="H26" s="3">
-        <v>2</v>
-      </c>
-      <c r="L26" t="s">
+      <c r="E23" s="4">
+        <v>2</v>
+      </c>
+      <c r="I23" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" customFormat="1" spans="5:14">
-      <c r="G27" s="2">
+    <row r="24" customFormat="1" spans="2:11">
+      <c r="D24" s="2">
         <v>1</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="E24" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M27" s="4">
+      <c r="J24" s="3">
         <v>0</v>
       </c>
-      <c r="N27" t="s">
+      <c r="K24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" customFormat="1" spans="5:14">
-      <c r="G28" s="2">
-        <v>2</v>
-      </c>
-      <c r="H28" s="3">
+    <row r="25" customFormat="1" spans="2:11">
+      <c r="D25" s="2">
+        <v>2</v>
+      </c>
+      <c r="E25" s="4">
         <v>1</v>
       </c>
-      <c r="M28" s="4">
+      <c r="J25" s="3">
         <v>4</v>
       </c>
-      <c r="N28" t="s">
+      <c r="K25" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" customFormat="1" spans="5:14">
-      <c r="G29" s="2">
+    <row r="26" customFormat="1" spans="2:11">
+      <c r="D26" s="2">
         <v>3</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="E26" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M29" s="4">
+      <c r="J26" s="3">
         <v>8</v>
       </c>
-      <c r="N29" t="s">
+      <c r="K26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" customFormat="1" spans="5:14">
-      <c r="G30" s="2">
+    <row r="27" customFormat="1" spans="2:11">
+      <c r="D27" s="2">
         <v>4</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="M30" s="4" t="s">
+      <c r="J27" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="N30" t="s">
+      <c r="K27" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="31" customFormat="1" spans="5:14">
-      <c r="G31" s="2">
+    <row r="28" customFormat="1" spans="2:11">
+      <c r="D28" s="2">
         <v>5</v>
       </c>
-      <c r="H31" s="3"/>
-      <c r="M31" s="4">
+      <c r="E28" s="4"/>
+      <c r="J28" s="3">
         <v>10</v>
       </c>
-      <c r="N31" t="s">
+      <c r="K28" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="32" customFormat="1" spans="5:14">
-      <c r="G32" s="2">
+    <row r="29" customFormat="1" spans="2:11">
+      <c r="D29" s="2">
         <v>6</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="E29" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M32" s="4">
+      <c r="J29" s="3">
         <v>14</v>
       </c>
-      <c r="N32" t="s">
+      <c r="K29" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="33" customFormat="1" spans="7:15">
-      <c r="G33" s="2">
+    <row r="30" customFormat="1" spans="2:11">
+      <c r="D30" s="2">
         <v>7</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="E30" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="M33" s="4">
+      <c r="J30" s="3">
         <v>18</v>
       </c>
-      <c r="N33" t="s">
+      <c r="K30" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="34" customFormat="1" spans="7:15">
-      <c r="G34" s="2">
+    <row r="31" customFormat="1" spans="2:11">
+      <c r="D31" s="2">
         <v>8</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="M34" s="4" t="s">
+      <c r="E31" s="4"/>
+      <c r="J31" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N34" t="s">
+      <c r="K31" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="35" customFormat="1" spans="7:15">
-      <c r="G35" s="2">
+    <row r="32" customFormat="1" spans="2:11">
+      <c r="D32" s="2">
         <v>9</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="E32" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="M35" s="4">
+      <c r="J32" s="3">
         <v>20</v>
       </c>
-      <c r="N35" t="s">
+      <c r="K32" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="36" customFormat="1" spans="7:15">
-      <c r="G36" s="2" t="s">
+    <row r="33" customFormat="1" spans="4:12">
+      <c r="D33" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="E33" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="M36" s="4">
+      <c r="J33" s="3">
         <v>24</v>
       </c>
-      <c r="N36" t="s">
+      <c r="K33" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" customFormat="1" spans="7:15">
-      <c r="G37" s="2" t="s">
+    <row r="34" customFormat="1" spans="4:12">
+      <c r="D34" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H37" s="3"/>
-      <c r="M37" s="4">
+      <c r="E34" s="4"/>
+      <c r="J34" s="3">
         <v>28</v>
       </c>
-      <c r="N37" t="s">
+      <c r="K34" t="s">
         <v>28</v>
       </c>
-      <c r="O37" t="s">
+      <c r="L34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="38" customFormat="1" spans="7:15">
-      <c r="G38" s="2" t="s">
+    <row r="35" customFormat="1" spans="4:12">
+      <c r="D35" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="E35" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L38" t="s">
+      <c r="I35" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="39" customFormat="1" spans="7:15">
-      <c r="G39" s="2" t="s">
+    <row r="36" customFormat="1" spans="4:12">
+      <c r="D36" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="3"/>
-    </row>
-    <row r="40" customFormat="1" spans="7:15">
-      <c r="G40" s="2" t="s">
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" customFormat="1" spans="4:12">
+      <c r="D37" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="E37" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2339,7 +2339,9 @@
       <c r="G26" s="2">
         <v>0</v>
       </c>
-      <c r="H26" s="3"/>
+      <c r="H26" t="s">
+        <v>10</v>
+      </c>
       <c r="L26" t="s">
         <v>6</v>
       </c>
@@ -2348,8 +2350,10 @@
       <c r="G27" s="2">
         <v>1</v>
       </c>
-      <c r="H27" s="3"/>
-      <c r="M27" s="4">
+      <c r="H27" t="s">
+        <v>15</v>
+      </c>
+      <c r="M27" s="3">
         <v>0</v>
       </c>
       <c r="N27" t="s">
@@ -2360,8 +2364,10 @@
       <c r="G28" s="2">
         <v>2</v>
       </c>
-      <c r="H28" s="3"/>
-      <c r="M28" s="4">
+      <c r="H28" t="s">
+        <v>12</v>
+      </c>
+      <c r="M28" s="3">
         <v>4</v>
       </c>
       <c r="N28" t="s">
@@ -2372,8 +2378,8 @@
       <c r="G29" s="2">
         <v>3</v>
       </c>
-      <c r="H29" s="3"/>
-      <c r="M29" s="4">
+      <c r="H29" s="4"/>
+      <c r="M29" s="3">
         <v>8</v>
       </c>
       <c r="N29" t="s">
@@ -2384,8 +2390,10 @@
       <c r="G30" s="2">
         <v>4</v>
       </c>
-      <c r="H30" s="3"/>
-      <c r="M30" s="4" t="s">
+      <c r="H30" t="s">
+        <v>23</v>
+      </c>
+      <c r="M30" s="3" t="s">
         <v>14</v>
       </c>
       <c r="N30" t="s">
@@ -2396,8 +2404,10 @@
       <c r="G31" s="2">
         <v>5</v>
       </c>
-      <c r="H31" s="3"/>
-      <c r="M31" s="4">
+      <c r="H31" t="s">
+        <v>17</v>
+      </c>
+      <c r="M31" s="3">
         <v>10</v>
       </c>
       <c r="N31" t="s">
@@ -2408,8 +2418,10 @@
       <c r="G32" s="2">
         <v>6</v>
       </c>
-      <c r="H32" s="3"/>
-      <c r="M32" s="4">
+      <c r="H32" t="s">
+        <v>26</v>
+      </c>
+      <c r="M32" s="3">
         <v>14</v>
       </c>
       <c r="N32" t="s">
@@ -2420,8 +2432,10 @@
       <c r="G33" s="2">
         <v>7</v>
       </c>
-      <c r="H33" s="3"/>
-      <c r="M33" s="4">
+      <c r="H33" t="s">
+        <v>19</v>
+      </c>
+      <c r="M33" s="3">
         <v>18</v>
       </c>
       <c r="N33" t="s">
@@ -2432,8 +2446,10 @@
       <c r="G34" s="2">
         <v>8</v>
       </c>
-      <c r="H34" s="3"/>
-      <c r="M34" s="4" t="s">
+      <c r="H34" t="s">
+        <v>21</v>
+      </c>
+      <c r="M34" s="3" t="s">
         <v>20</v>
       </c>
       <c r="N34" t="s">
@@ -2444,8 +2460,8 @@
       <c r="G35" s="2">
         <v>9</v>
       </c>
-      <c r="H35" s="3"/>
-      <c r="M35" s="4">
+      <c r="H35" s="4"/>
+      <c r="M35" s="3">
         <v>20</v>
       </c>
       <c r="N35" t="s">
@@ -2456,8 +2472,8 @@
       <c r="G36" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H36" s="3"/>
-      <c r="M36" s="4">
+      <c r="H36" s="4"/>
+      <c r="M36" s="3">
         <v>24</v>
       </c>
       <c r="N36" t="s">
@@ -2468,8 +2484,8 @@
       <c r="G37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H37" s="3"/>
-      <c r="M37" s="4">
+      <c r="H37" s="4"/>
+      <c r="M37" s="3">
         <v>28</v>
       </c>
       <c r="N37" t="s">
@@ -2483,7 +2499,9 @@
       <c r="G38" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H38" s="3"/>
+      <c r="H38" t="s">
+        <v>9</v>
+      </c>
       <c r="L38" t="s">
         <v>8</v>
       </c>
@@ -2492,13 +2510,13 @@
       <c r="G39" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H39" s="3"/>
+      <c r="H39" s="4"/>
     </row>
     <row r="40" customFormat="1" spans="7:15">
       <c r="G40" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H40" s="3"/>
+      <c r="H40" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>